<commit_message>
fix(excel): make template header visible (white bold on navy fill)
The header row used a bold font with no explicit color, which resolved to an
invisible/white color in some Excel themes. Now the header uses an explicit
white bold font on a solid navy fill with a bottom border, so it is clearly
visible in any theme. Regenerated both sample files to match.
</commit_message>
<xml_diff>
--- a/docs/sample-data/Sample_MCQs_for_upload.xlsx
+++ b/docs/sample-data/Sample_MCQs_for_upload.xlsx
@@ -7,51 +7,97 @@
 </workbook>
 </file>
 
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+  </fonts>
+  <fills count="3">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A2B4A"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+  </cellXfs>
+</styleSheet>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Stack_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Topic_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Difficulty</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Question_Stem</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Option_A</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Option_B</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Option_C</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Option_D</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Correct_answer</t>
         </is>

</xml_diff>